<commit_message>
add more layers to config examples and make consistent between json and .xlsx
</commit_message>
<xml_diff>
--- a/examples/configuration_templates/pfa_config_example.xlsx
+++ b/examples/configuration_templates/pfa_config_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smello\code\geoPFA\examples\configuration_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A1C1C7-1115-40B4-94F9-6187D3C636A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E5CA54-7A5B-4D32-B982-624767AB3F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37305" yWindow="-8775" windowWidth="18000" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="1080" windowWidth="18288" windowHeight="11028" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="44">
   <si>
     <t>criteria</t>
   </si>
@@ -127,6 +127,36 @@
   </si>
   <si>
     <t>Geometry-only shapefile; coordinate columns are omitted.</t>
+  </si>
+  <si>
+    <t>economic</t>
+  </si>
+  <si>
+    <t>demand</t>
+  </si>
+  <si>
+    <t>infrastructure</t>
+  </si>
+  <si>
+    <t>dist_to_roads</t>
+  </si>
+  <si>
+    <t>dist_to_transmission</t>
+  </si>
+  <si>
+    <t>electricity_price</t>
+  </si>
+  <si>
+    <t>km</t>
+  </si>
+  <si>
+    <t>$/kWh</t>
+  </si>
+  <si>
+    <t>dist</t>
+  </si>
+  <si>
+    <t>cost</t>
   </si>
 </sst>
 </file>
@@ -466,15 +496,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
     <col min="2" max="2" width="14.109375" customWidth="1"/>
     <col min="3" max="3" width="13.109375" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="6" max="7" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" customWidth="1"/>
     <col min="9" max="9" width="8.33203125" customWidth="1"/>
-    <col min="16" max="16" width="12.33203125" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="15" max="16" width="12.33203125" customWidth="1"/>
+    <col min="17" max="17" width="32.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -535,7 +569,7 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -616,6 +650,117 @@
       </c>
       <c r="Q3" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4">
+        <v>0.5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4">
+        <v>0.7</v>
+      </c>
+      <c r="E4">
+        <v>0.25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4">
+        <v>0.6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5">
+        <v>0.4</v>
+      </c>
+      <c r="H5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6">
+        <v>0.3</v>
+      </c>
+      <c r="E6">
+        <v>0.1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" t="s">
+        <v>31</v>
+      </c>
+      <c r="P6" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>